<commit_message>
Bug Fix and nigeria add
</commit_message>
<xml_diff>
--- a/UserScore/MonthlyUserScore.xlsx
+++ b/UserScore/MonthlyUserScore.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F915"/>
+  <dimension ref="A1:F916"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24224,6 +24224,32 @@
         <v>2</v>
       </c>
     </row>
+    <row r="916">
+      <c r="A916" t="n">
+        <v>915</v>
+      </c>
+      <c r="B916" t="inlineStr">
+        <is>
+          <t>-1002359766306</t>
+        </is>
+      </c>
+      <c r="C916" t="inlineStr">
+        <is>
+          <t>5080276560</t>
+        </is>
+      </c>
+      <c r="D916" t="inlineStr">
+        <is>
+          <t>@BhaKth_bH0lenath_ka</t>
+        </is>
+      </c>
+      <c r="E916" t="n">
+        <v>3</v>
+      </c>
+      <c r="F916" t="n">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
updated and add Quizzes
</commit_message>
<xml_diff>
--- a/UserScore/MonthlyUserScore.xlsx
+++ b/UserScore/MonthlyUserScore.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F603"/>
+  <dimension ref="A1:F605"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16112,6 +16112,58 @@
         <v>1</v>
       </c>
     </row>
+    <row r="604">
+      <c r="A604" t="n">
+        <v>603</v>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>5080276560</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>5080276560</t>
+        </is>
+      </c>
+      <c r="D604" t="inlineStr">
+        <is>
+          <t>@BhaKth_bH0lenath_ka</t>
+        </is>
+      </c>
+      <c r="E604" t="n">
+        <v>5</v>
+      </c>
+      <c r="F604" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="n">
+        <v>604</v>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>-1002359766306</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>5080276560</t>
+        </is>
+      </c>
+      <c r="D605" t="inlineStr">
+        <is>
+          <t>@BhaKth_bH0lenath_ka</t>
+        </is>
+      </c>
+      <c r="E605" t="n">
+        <v>2</v>
+      </c>
+      <c r="F605" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>